<commit_message>
Enhance Playwright framework with encrypted test data
</commit_message>
<xml_diff>
--- a/test-data/userData.xlsx
+++ b/test-data/userData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/priyanshu/PROJECTS/Playwright_Automation/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{125BC0E9-CE26-D442-980C-9479F5D760C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CEE8AB4-617E-9C45-943C-20AD032E086A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16900" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -24,12 +24,50 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
+  <si>
+    <t>executor</t>
+  </si>
+  <si>
+    <t>TestCase_ID</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>TC02pro</t>
+  </si>
+  <si>
+    <t>TC01prod</t>
+  </si>
+  <si>
+    <t>PAN</t>
+  </si>
+  <si>
+    <t>Aadhaar</t>
+  </si>
+  <si>
+    <t>43e5c2081091ac121c4357ed:6e1425846d05f71692f1d80bca6c9b8c:b3b0979116506e532060</t>
+  </si>
+  <si>
+    <t>ec62aa977b983f2bce728e93:87440ea64f7ef762174c01b4614d0d3c:fef44ea2547ba64d25ad6eef</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -318,9 +356,57 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{682EB8EF-2246-4946-8DA5-364EE65A7DA0}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="3" max="3" width="78.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="81.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>